<commit_message>
fix: centrar descripcion en excel
</commit_message>
<xml_diff>
--- a/ModuloWeb1/bin/Debug/net10.0/Ordenes/4-0.xlsx
+++ b/ModuloWeb1/bin/Debug/net10.0/Ordenes/4-0.xlsx
@@ -5,10 +5,10 @@
   <x:workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\milo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\milo\moduloweb-ordenes-compra\ModuloWeb1\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7858ACF5-2E4C-425E-9D04-03D4F7C32F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086B9B91-C8D3-4E46-AAC5-F36A31431B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -28,12 +28,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t>Estado de orden:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Proveedor: ABB_COLOMBIA_LTDA</x:t>
-  </x:si>
   <x:si>
     <x:r>
       <x:rPr>
@@ -195,13 +189,13 @@
     <x:t>Item</x:t>
   </x:si>
   <x:si>
-    <x:t>Catalogo</x:t>
+    <x:t xml:space="preserve">Descripcion </x:t>
   </x:si>
   <x:si>
     <x:t>Modelo</x:t>
   </x:si>
   <x:si>
-    <x:t>Descripcion</x:t>
+    <x:t>N° Catálogo</x:t>
   </x:si>
   <x:si>
     <x:t>F. Entrega</x:t>
@@ -258,7 +252,7 @@
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>13/03/2026</x:t>
+    <x:t>07/04/2026</x:t>
   </x:si>
   <x:si>
     <x:t>NA</x:t>
@@ -273,19 +267,34 @@
     <x:t>4</x:t>
   </x:si>
   <x:si>
-    <x:t>TOTAL:</x:t>
+    <x:t>Subtotal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Firma y sello</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Observaciones:</x:t>
   </x:si>
   <x:si>
     <x:t>UND</x:t>
   </x:si>
   <x:si>
-    <x:t>432</x:t>
+    <x:t>REF. HD100P1ES MOTOR US MOTORS NEMA PREMIUM 100 HP @ 3600 RPM FRAME 405TS</x:t>
   </x:si>
   <x:si>
     <x:t>4-0</x:t>
   </x:si>
   <x:si>
     <x:t>COP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IVA:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total:</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -301,7 +310,7 @@
     <x:numFmt numFmtId="169" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <x:numFmt numFmtId="170" formatCode="#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF000000"/>
@@ -370,10 +379,33 @@
       <x:name val="Docs-Roboto"/>
     </x:font>
     <x:font>
+      <x:u/>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
       <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="9"/>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
       <x:family val="2"/>
     </x:font>
   </x:fonts>
@@ -403,27 +435,12 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="33">
+  <x:borders count="36">
     <x:border>
       <x:left/>
       <x:right/>
       <x:top/>
       <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
       <x:diagonal/>
     </x:border>
     <x:border>
@@ -721,6 +738,23 @@
       <x:left style="thin">
         <x:color rgb="FF000000"/>
       </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
       <x:right style="medium">
         <x:color rgb="FF000000"/>
       </x:right>
@@ -741,7 +775,7 @@
       <x:right style="none">
         <x:color rgb="FF000000"/>
       </x:right>
-      <x:top style="none">
+      <x:top style="thin">
         <x:color rgb="FF000000"/>
       </x:top>
       <x:bottom style="medium">
@@ -758,7 +792,7 @@
       <x:right style="none">
         <x:color rgb="FF000000"/>
       </x:right>
-      <x:top style="none">
+      <x:top style="thin">
         <x:color rgb="FF000000"/>
       </x:top>
       <x:bottom style="medium">
@@ -772,10 +806,61 @@
       <x:left style="none">
         <x:color rgb="FF000000"/>
       </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="none">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
       <x:right style="medium">
         <x:color rgb="FF000000"/>
       </x:right>
-      <x:top style="none">
+      <x:top style="thin">
         <x:color rgb="FF000000"/>
       </x:top>
       <x:bottom style="medium">
@@ -786,12 +871,12 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="53">
+  <x:cellStyleXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -803,58 +888,61 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="5" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="11" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="12" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="13" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="16" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="7" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="20" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="6" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="19" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="22" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="20" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="20" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="19" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="19" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="24" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="25" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -863,40 +951,43 @@
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="26" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="27" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="27" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="14" fontId="3" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="170" fontId="3" fillId="0" borderId="29" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="30" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="30" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="31" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="166" fontId="3" fillId="0" borderId="31" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="31" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="170" fontId="6" fillId="0" borderId="32" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="32" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="33" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="34" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="35" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -905,15 +996,30 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="19" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="21" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="170" fontId="10" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="21" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="170" fontId="6" fillId="0" borderId="28" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -945,11 +1051,9 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="114">
+  <x:cellXfs count="127">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
@@ -957,13 +1061,13 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1090,84 +1194,92 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
+    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1179,16 +1291,20 @@
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="3" fontId="8" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1199,31 +1315,31 @@
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="14" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="165" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1231,27 +1347,67 @@
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="166" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="170" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="170" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="170" fontId="6" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="170" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1269,22 +1425,22 @@
   </x:cellStyles>
   <x:tableStyles count="3">
     <x:tableStyle name="info-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <x:tableStyleElement type="wholeTable" size="0" dxfId="8"/>
-      <x:tableStyleElement type="headerRow" dxfId="11"/>
-      <x:tableStyleElement type="firstRowStripe" dxfId="10"/>
-      <x:tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <x:tableStyleElement type="wholeTable" size="0" dxfId="11"/>
+      <x:tableStyleElement type="headerRow" dxfId="10"/>
+      <x:tableStyleElement type="firstRowStripe" dxfId="9"/>
+      <x:tableStyleElement type="secondRowStripe" dxfId="8"/>
     </x:tableStyle>
     <x:tableStyle name="forms_productos-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <x:tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <x:tableStyleElement type="headerRow" dxfId="7"/>
-      <x:tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <x:tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <x:tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <x:tableStyleElement type="headerRow" dxfId="6"/>
+      <x:tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <x:tableStyleElement type="secondRowStripe" dxfId="4"/>
     </x:tableStyle>
     <x:tableStyle name="forms-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <x:tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <x:tableStyleElement type="headerRow" dxfId="3"/>
-      <x:tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <x:tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <x:tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <x:tableStyleElement type="headerRow" dxfId="2"/>
+      <x:tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <x:tableStyleElement type="secondRowStripe" dxfId="0"/>
     </x:tableStyle>
   </x:tableStyles>
   <x:extLst>
@@ -1542,7 +1698,7 @@
     <x:col min="1" max="1" width="2.726562" style="0" customWidth="1"/>
     <x:col min="2" max="3" width="5" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="13.632812" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="32.726562" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38.179688" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="25.453125" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="19" style="0" customWidth="1"/>
@@ -1559,155 +1715,153 @@
       <x:c r="M1" s="1"/>
     </x:row>
     <x:row r="2" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="L2" s="2" t="s">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="L2" s="50"/>
     </x:row>
     <x:row r="3" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="L3" s="2"/>
+      <x:c r="L3" s="50"/>
     </x:row>
     <x:row r="4" spans="1:26" ht="12.75" customHeight="1"/>
-    <x:row r="5" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="L5" s="4"/>
-    </x:row>
-    <x:row r="6" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="I6" s="5">
+    <x:row r="5" spans="1:26" ht="12.5" customHeight="1">
+      <x:c r="L5" s="2"/>
+    </x:row>
+    <x:row r="6" spans="1:26" ht="19.5" customHeight="1">
+      <x:c r="I6" s="3">
         <x:f>"ORDEN DE COMPRA No: "</x:f>
       </x:c>
-      <x:c r="J6" s="5"/>
-      <x:c r="K6" s="5"/>
-      <x:c r="L6" s="5"/>
-      <x:c r="M6" s="6">
+      <x:c r="J6" s="3"/>
+      <x:c r="K6" s="3"/>
+      <x:c r="L6" s="3"/>
+      <x:c r="M6" s="4">
         <x:f>Instancia!B2</x:f>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:26" ht="6.75" customHeight="1"/>
     <x:row r="8" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B8" s="87" t="s">
-        <x:v>1</x:v>
+      <x:c r="B8" s="89">
+        <x:f>"Proveedor: " &amp; Instancia!L2</x:f>
       </x:c>
       <x:c r="C8" s="57"/>
       <x:c r="D8" s="57"/>
       <x:c r="E8" s="57"/>
       <x:c r="F8" s="57"/>
       <x:c r="G8" s="57"/>
-      <x:c r="H8" s="88"/>
-      <x:c r="J8" s="87" t="s">
-        <x:v>2</x:v>
+      <x:c r="H8" s="90"/>
+      <x:c r="J8" s="89" t="s">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K8" s="57"/>
       <x:c r="L8" s="57"/>
       <x:c r="M8" s="57"/>
-      <x:c r="N8" s="89"/>
+      <x:c r="N8" s="91"/>
     </x:row>
     <x:row r="9" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B9" s="90">
+      <x:c r="B9" s="92">
         <x:f>"NIT/CC: " &amp; Instancia!M2</x:f>
       </x:c>
-      <x:c r="C9" s="91"/>
-      <x:c r="D9" s="91"/>
-      <x:c r="E9" s="91"/>
-      <x:c r="F9" s="91"/>
-      <x:c r="G9" s="91"/>
+      <x:c r="C9" s="93"/>
+      <x:c r="D9" s="93"/>
+      <x:c r="E9" s="93"/>
+      <x:c r="F9" s="93"/>
+      <x:c r="G9" s="93"/>
       <x:c r="H9" s="62"/>
-      <x:c r="J9" s="90" t="s">
+      <x:c r="J9" s="92" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K9" s="93"/>
+      <x:c r="L9" s="93"/>
+      <x:c r="M9" s="93"/>
+      <x:c r="N9" s="62"/>
+    </x:row>
+    <x:row r="10" spans="1:26" ht="12.75" customHeight="1">
+      <x:c r="B10" s="92">
+        <x:f>"Ciudad: " &amp; Instancia!N2</x:f>
+      </x:c>
+      <x:c r="C10" s="93"/>
+      <x:c r="D10" s="93"/>
+      <x:c r="E10" s="93"/>
+      <x:c r="F10" s="93"/>
+      <x:c r="G10" s="93"/>
+      <x:c r="H10" s="62"/>
+      <x:c r="J10" s="92" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K10" s="93"/>
+      <x:c r="L10" s="93"/>
+      <x:c r="M10" s="93"/>
+      <x:c r="N10" s="62"/>
+    </x:row>
+    <x:row r="11" spans="1:26" ht="12.75" customHeight="1">
+      <x:c r="B11" s="92">
+        <x:f>"Dirección: " &amp; Instancia!O2</x:f>
+      </x:c>
+      <x:c r="C11" s="93"/>
+      <x:c r="D11" s="93"/>
+      <x:c r="E11" s="93"/>
+      <x:c r="F11" s="93"/>
+      <x:c r="G11" s="93"/>
+      <x:c r="H11" s="62"/>
+      <x:c r="J11" s="92" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K9" s="91"/>
-      <x:c r="L9" s="91"/>
-      <x:c r="M9" s="91"/>
-      <x:c r="N9" s="62"/>
-    </x:row>
-    <x:row r="10" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B10" s="90">
-        <x:f>"Ciudad: " &amp; Instancia!N2</x:f>
-      </x:c>
-      <x:c r="C10" s="91"/>
-      <x:c r="D10" s="91"/>
-      <x:c r="E10" s="91"/>
-      <x:c r="F10" s="91"/>
-      <x:c r="G10" s="91"/>
-      <x:c r="H10" s="62"/>
-      <x:c r="J10" s="90" t="s">
+      <x:c r="K11" s="93"/>
+      <x:c r="L11" s="93"/>
+      <x:c r="M11" s="93"/>
+      <x:c r="N11" s="62"/>
+    </x:row>
+    <x:row r="12" spans="1:26" ht="12.75" customHeight="1" hidden="1">
+      <x:c r="B12" s="92" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K10" s="91"/>
-      <x:c r="L10" s="91"/>
-      <x:c r="M10" s="91"/>
-      <x:c r="N10" s="62"/>
-    </x:row>
-    <x:row r="11" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B11" s="90">
-        <x:f>"Dirección: " &amp; Instancia!O2</x:f>
-      </x:c>
-      <x:c r="C11" s="91"/>
-      <x:c r="D11" s="91"/>
-      <x:c r="E11" s="91"/>
-      <x:c r="F11" s="91"/>
-      <x:c r="G11" s="91"/>
-      <x:c r="H11" s="62"/>
-      <x:c r="J11" s="90" t="s">
+      <x:c r="C12" s="93"/>
+      <x:c r="D12" s="93"/>
+      <x:c r="E12" s="93"/>
+      <x:c r="F12" s="93"/>
+      <x:c r="G12" s="93"/>
+      <x:c r="H12" s="62"/>
+      <x:c r="J12" s="92" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K11" s="91"/>
-      <x:c r="L11" s="91"/>
-      <x:c r="M11" s="91"/>
-      <x:c r="N11" s="62"/>
-    </x:row>
-    <x:row r="12" spans="1:26" ht="12.75" customHeight="1" hidden="1">
-      <x:c r="B12" s="90" t="s">
+      <x:c r="K12" s="93"/>
+      <x:c r="L12" s="93"/>
+      <x:c r="M12" s="94" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C12" s="91"/>
-      <x:c r="D12" s="91"/>
-      <x:c r="E12" s="91"/>
-      <x:c r="F12" s="91"/>
-      <x:c r="G12" s="91"/>
-      <x:c r="H12" s="62"/>
-      <x:c r="J12" s="90" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="K12" s="91"/>
-      <x:c r="L12" s="91"/>
-      <x:c r="M12" s="92" t="s">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="N12" s="62"/>
     </x:row>
     <x:row r="13" spans="1:26" ht="22.5" customHeight="1">
-      <x:c r="B13" s="93">
+      <x:c r="B13" s="95">
         <x:f>"Contacto: " &amp; Instancia!C2</x:f>
       </x:c>
       <x:c r="C13" s="66"/>
       <x:c r="D13" s="66"/>
       <x:c r="E13" s="66"/>
-      <x:c r="F13" s="94"/>
+      <x:c r="F13" s="96"/>
       <x:c r="G13" s="66"/>
       <x:c r="H13" s="69"/>
-      <x:c r="J13" s="95" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="K13" s="91"/>
-      <x:c r="L13" s="91"/>
-      <x:c r="M13" s="91"/>
+      <x:c r="J13" s="97" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K13" s="93"/>
+      <x:c r="L13" s="93"/>
+      <x:c r="M13" s="93"/>
       <x:c r="N13" s="62"/>
     </x:row>
     <x:row r="14" spans="1:26" ht="12.75" customHeight="1">
       <x:c r="B14" s="73" t="s">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="74"/>
       <x:c r="D14" s="75"/>
       <x:c r="E14" s="73" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F14" s="75"/>
       <x:c r="G14" s="73" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H14" s="74"/>
       <x:c r="I14" s="75"/>
-      <x:c r="J14" s="84">
+      <x:c r="J14" s="81">
         <x:f>"Entregar a Alterno: " &amp; Instancia!H2</x:f>
       </x:c>
       <x:c r="K14" s="74"/>
@@ -1716,21 +1870,21 @@
       <x:c r="N14" s="75"/>
     </x:row>
     <x:row r="15" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B15" s="78">
+      <x:c r="B15" s="85">
         <x:f>Instancia!E2</x:f>
       </x:c>
       <x:c r="C15" s="74"/>
       <x:c r="D15" s="75"/>
-      <x:c r="E15" s="79">
+      <x:c r="E15" s="86">
         <x:f>Instancia!F2</x:f>
       </x:c>
       <x:c r="F15" s="75"/>
-      <x:c r="G15" s="79">
+      <x:c r="G15" s="86">
         <x:f>Instancia!P2</x:f>
       </x:c>
       <x:c r="H15" s="74"/>
       <x:c r="I15" s="75"/>
-      <x:c r="J15" s="84">
+      <x:c r="J15" s="81">
         <x:f>"Entregar a: " &amp; Instancia!G2</x:f>
       </x:c>
       <x:c r="K15" s="74"/>
@@ -1739,7 +1893,7 @@
       <x:c r="N15" s="75"/>
     </x:row>
     <x:row r="16" spans="1:26" ht="12.75" customHeight="1">
-      <x:c r="B16" s="85">
+      <x:c r="B16" s="82">
         <x:f>"Condiciones de pago: " &amp; Instancia!I2</x:f>
       </x:c>
       <x:c r="C16" s="74"/>
@@ -1757,496 +1911,514 @@
     </x:row>
     <x:row r="17" spans="1:26" ht="22.5" customHeight="1"/>
     <x:row r="18" spans="1:26" ht="24.75" customHeight="1">
-      <x:c r="B18" s="96" t="s">
+      <x:c r="B18" s="98" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C18" s="99"/>
+      <x:c r="D18" s="99" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E18" s="99" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C18" s="97"/>
-      <x:c r="D18" s="97" t="s">
+      <x:c r="F18" s="99" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E18" s="97" t="s">
+      <x:c r="G18" s="99" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F18" s="97" t="s">
+      <x:c r="H18" s="99" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G18" s="97" t="s">
+      <x:c r="I18" s="99" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H18" s="97" t="s">
+      <x:c r="J18" s="99" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I18" s="97" t="s">
+      <x:c r="K18" s="99" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J18" s="97" t="s">
+      <x:c r="L18" s="99" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K18" s="97" t="s">
+      <x:c r="M18" s="99" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="L18" s="97" t="s">
+      <x:c r="N18" s="100" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M18" s="97" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N18" s="98" t="s">
-        <x:v>24</x:v>
-      </x:c>
     </x:row>
     <x:row r="19" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B19" s="99">
+      <x:c r="B19" s="101">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C19" s="100"/>
-      <x:c r="D19" s="101" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E19" s="100" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F19" s="100" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="G19" s="102" t="s">
+      <x:c r="C19" s="102"/>
+      <x:c r="D19" s="103" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E19" s="104" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="H19" s="103" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="I19" s="100">
+      <x:c r="F19" s="102" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="G19" s="105" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H19" s="106" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I19" s="102">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J19" s="100">
+      <x:c r="J19" s="102">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K19" s="100" t="s">
+      <x:c r="K19" s="102" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="L19" s="104">
-        <x:v>432</x:v>
-      </x:c>
-      <x:c r="M19" s="100">
+      <x:c r="L19" s="107">
+        <x:v>21089572.06</x:v>
+      </x:c>
+      <x:c r="M19" s="102">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N19" s="105">
+      <x:c r="N19" s="108">
         <x:f>J19*L19*(1-(M19/100))*(1+(I19/100))</x:f>
       </x:c>
     </x:row>
-    <x:row r="20" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B20" s="106"/>
-      <x:c r="C20" s="107"/>
-      <x:c r="D20" s="107"/>
-      <x:c r="E20" s="108"/>
-      <x:c r="F20" s="107"/>
-      <x:c r="G20" s="108"/>
-      <x:c r="H20" s="108"/>
-      <x:c r="I20" s="107"/>
-      <x:c r="J20" s="107"/>
-      <x:c r="K20" s="107"/>
-      <x:c r="L20" s="109"/>
-      <x:c r="M20" s="110" t="s">
+    <x:row r="20" spans="1:26" ht="50" customHeight="1">
+      <x:c r="B20" s="109" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="N20" s="111">
-        <x:f>SUM(N19:N19)</x:f>
-      </x:c>
-    </x:row>
-    <x:row r="21" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B21" s="10"/>
-      <x:c r="C21" s="10"/>
-      <x:c r="D21" s="10"/>
-      <x:c r="E21" s="19"/>
-      <x:c r="F21" s="19"/>
-      <x:c r="G21" s="19"/>
-      <x:c r="H21" s="19"/>
-      <x:c r="I21" s="19"/>
-      <x:c r="J21" s="19"/>
-      <x:c r="K21" s="19"/>
-      <x:c r="L21" s="19"/>
-      <x:c r="M21" s="19"/>
-      <x:c r="N21" s="19"/>
-    </x:row>
-    <x:row r="22" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B22" s="10"/>
-      <x:c r="C22" s="10"/>
-      <x:c r="D22" s="10"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="10"/>
-      <x:c r="G22" s="10"/>
-      <x:c r="H22" s="10"/>
-      <x:c r="I22" s="10"/>
-      <x:c r="J22" s="10"/>
-      <x:c r="K22" s="10"/>
-      <x:c r="L22" s="10"/>
-      <x:c r="M22" s="14"/>
-      <x:c r="N22" s="14"/>
+      <x:c r="C20" s="110"/>
+      <x:c r="D20" s="110"/>
+      <x:c r="E20" s="110"/>
+      <x:c r="F20" s="110"/>
+      <x:c r="G20" s="111"/>
+      <x:c r="H20" s="112" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="I20" s="110"/>
+      <x:c r="J20" s="111"/>
+      <x:c r="K20" s="113" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="L20" s="114"/>
+      <x:c r="M20" s="115" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="N20" s="116">
+        <x:v>21089572.06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:26" ht="15" customHeight="1">
+      <x:c r="B21" s="8"/>
+      <x:c r="C21" s="8"/>
+      <x:c r="D21" s="8"/>
+      <x:c r="E21" s="17"/>
+      <x:c r="F21" s="17"/>
+      <x:c r="G21" s="17"/>
+      <x:c r="H21" s="17"/>
+      <x:c r="I21" s="17"/>
+      <x:c r="J21" s="17"/>
+      <x:c r="K21" s="117" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="L21" s="118"/>
+      <x:c r="M21" s="119" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="N21" s="120">
+        <x:v>4007018.6914</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:26" ht="15" customHeight="1">
+      <x:c r="B22" s="8"/>
+      <x:c r="C22" s="8"/>
+      <x:c r="D22" s="8"/>
+      <x:c r="E22" s="12"/>
+      <x:c r="F22" s="8"/>
+      <x:c r="G22" s="8"/>
+      <x:c r="H22" s="8"/>
+      <x:c r="I22" s="8"/>
+      <x:c r="J22" s="8"/>
+      <x:c r="K22" s="121" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="L22" s="122"/>
+      <x:c r="M22" s="123" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="N22" s="124">
+        <x:v>25096590.7514</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B23" s="10"/>
-      <x:c r="C23" s="10"/>
-      <x:c r="D23" s="10"/>
-      <x:c r="E23" s="14"/>
-      <x:c r="F23" s="10"/>
-      <x:c r="G23" s="14"/>
-      <x:c r="H23" s="14"/>
-      <x:c r="I23" s="10"/>
-      <x:c r="J23" s="10"/>
-      <x:c r="K23" s="10"/>
-      <x:c r="L23" s="16"/>
-      <x:c r="M23" s="14"/>
-      <x:c r="N23" s="18"/>
-      <x:c r="O23" s="20"/>
+      <x:c r="B23" s="8"/>
+      <x:c r="C23" s="8"/>
+      <x:c r="D23" s="8"/>
+      <x:c r="E23" s="12"/>
+      <x:c r="F23" s="8"/>
+      <x:c r="G23" s="12"/>
+      <x:c r="H23" s="12"/>
+      <x:c r="I23" s="8"/>
+      <x:c r="J23" s="8"/>
+      <x:c r="K23" s="8"/>
+      <x:c r="L23" s="14"/>
+      <x:c r="M23" s="12"/>
+      <x:c r="N23" s="16"/>
+      <x:c r="O23" s="18"/>
     </x:row>
     <x:row r="24" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B24" s="10"/>
-      <x:c r="C24" s="10"/>
-      <x:c r="D24" s="10"/>
-      <x:c r="E24" s="14"/>
-      <x:c r="F24" s="21"/>
-      <x:c r="G24" s="21"/>
-      <x:c r="H24" s="21"/>
-      <x:c r="I24" s="21"/>
-      <x:c r="J24" s="21"/>
-      <x:c r="K24" s="21"/>
-      <x:c r="L24" s="21"/>
-      <x:c r="M24" s="23"/>
-      <x:c r="N24" s="23"/>
+      <x:c r="B24" s="8"/>
+      <x:c r="C24" s="8"/>
+      <x:c r="D24" s="8"/>
+      <x:c r="E24" s="12"/>
+      <x:c r="F24" s="19"/>
+      <x:c r="G24" s="19"/>
+      <x:c r="H24" s="19"/>
+      <x:c r="I24" s="19"/>
+      <x:c r="J24" s="19"/>
+      <x:c r="K24" s="19"/>
+      <x:c r="L24" s="19"/>
+      <x:c r="M24" s="21"/>
+      <x:c r="N24" s="21"/>
     </x:row>
     <x:row r="25" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B25" s="10"/>
-      <x:c r="C25" s="10"/>
-      <x:c r="D25" s="10"/>
-      <x:c r="E25" s="14"/>
-      <x:c r="F25" s="10"/>
-      <x:c r="G25" s="25"/>
-      <x:c r="H25" s="14"/>
-      <x:c r="I25" s="10"/>
-      <x:c r="J25" s="10"/>
-      <x:c r="K25" s="26"/>
-      <x:c r="L25" s="27"/>
-      <x:c r="M25" s="28"/>
-      <x:c r="N25" s="29"/>
+      <x:c r="B25" s="8"/>
+      <x:c r="C25" s="8"/>
+      <x:c r="D25" s="8"/>
+      <x:c r="E25" s="12"/>
+      <x:c r="F25" s="8"/>
+      <x:c r="G25" s="23"/>
+      <x:c r="H25" s="12"/>
+      <x:c r="I25" s="8"/>
+      <x:c r="J25" s="8"/>
+      <x:c r="K25" s="24"/>
+      <x:c r="L25" s="25"/>
+      <x:c r="M25" s="26"/>
+      <x:c r="N25" s="27"/>
     </x:row>
     <x:row r="26" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B26" s="30"/>
-      <x:c r="C26" s="30"/>
-      <x:c r="D26" s="10"/>
-      <x:c r="E26" s="14"/>
-      <x:c r="F26" s="10"/>
-      <x:c r="G26" s="14"/>
-      <x:c r="H26" s="14"/>
-      <x:c r="I26" s="10"/>
-      <x:c r="J26" s="10"/>
-      <x:c r="K26" s="26"/>
-      <x:c r="L26" s="27"/>
-      <x:c r="M26" s="28"/>
-      <x:c r="N26" s="32"/>
+      <x:c r="B26" s="28"/>
+      <x:c r="C26" s="28"/>
+      <x:c r="D26" s="8"/>
+      <x:c r="E26" s="12"/>
+      <x:c r="F26" s="8"/>
+      <x:c r="G26" s="12"/>
+      <x:c r="H26" s="12"/>
+      <x:c r="I26" s="8"/>
+      <x:c r="J26" s="8"/>
+      <x:c r="K26" s="24"/>
+      <x:c r="L26" s="25"/>
+      <x:c r="M26" s="26"/>
+      <x:c r="N26" s="30"/>
     </x:row>
     <x:row r="27" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B27" s="30"/>
-      <x:c r="C27" s="30"/>
-      <x:c r="D27" s="10"/>
-      <x:c r="E27" s="14"/>
-      <x:c r="F27" s="10"/>
-      <x:c r="G27" s="14"/>
-      <x:c r="H27" s="14"/>
-      <x:c r="I27" s="10"/>
-      <x:c r="J27" s="10"/>
-      <x:c r="K27" s="26"/>
-      <x:c r="L27" s="27"/>
-      <x:c r="M27" s="28"/>
-      <x:c r="N27" s="32"/>
+      <x:c r="B27" s="28"/>
+      <x:c r="C27" s="28"/>
+      <x:c r="D27" s="8"/>
+      <x:c r="E27" s="12"/>
+      <x:c r="F27" s="8"/>
+      <x:c r="G27" s="12"/>
+      <x:c r="H27" s="12"/>
+      <x:c r="I27" s="8"/>
+      <x:c r="J27" s="8"/>
+      <x:c r="K27" s="24"/>
+      <x:c r="L27" s="25"/>
+      <x:c r="M27" s="26"/>
+      <x:c r="N27" s="30"/>
     </x:row>
     <x:row r="28" spans="1:26" ht="112.5" customHeight="1" hidden="1">
-      <x:c r="B28" s="30"/>
-      <x:c r="C28" s="30"/>
-      <x:c r="D28" s="10"/>
-      <x:c r="E28" s="14"/>
-      <x:c r="F28" s="10"/>
-      <x:c r="G28" s="14"/>
-      <x:c r="H28" s="14"/>
-      <x:c r="I28" s="10"/>
-      <x:c r="J28" s="10"/>
-      <x:c r="K28" s="26"/>
-      <x:c r="L28" s="36"/>
-      <x:c r="M28" s="28"/>
-      <x:c r="N28" s="37"/>
+      <x:c r="B28" s="28"/>
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="8"/>
+      <x:c r="E28" s="12"/>
+      <x:c r="F28" s="8"/>
+      <x:c r="G28" s="12"/>
+      <x:c r="H28" s="12"/>
+      <x:c r="I28" s="8"/>
+      <x:c r="J28" s="8"/>
+      <x:c r="K28" s="24"/>
+      <x:c r="L28" s="34"/>
+      <x:c r="M28" s="26"/>
+      <x:c r="N28" s="35"/>
     </x:row>
     <x:row r="29" spans="1:26" ht="112.5" customHeight="1" hidden="1">
-      <x:c r="B29" s="30"/>
-      <x:c r="C29" s="30"/>
-      <x:c r="K29" s="26"/>
-      <x:c r="M29" s="28"/>
+      <x:c r="B29" s="28"/>
+      <x:c r="C29" s="28"/>
+      <x:c r="K29" s="24"/>
+      <x:c r="M29" s="26"/>
     </x:row>
     <x:row r="30" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B30" s="30"/>
-      <x:c r="C30" s="30"/>
-      <x:c r="D30" s="10"/>
-      <x:c r="E30" s="14"/>
-      <x:c r="F30" s="10"/>
-      <x:c r="G30" s="14"/>
-      <x:c r="H30" s="14"/>
-      <x:c r="I30" s="10"/>
-      <x:c r="J30" s="10"/>
-      <x:c r="K30" s="26"/>
-      <x:c r="L30" s="27"/>
-      <x:c r="M30" s="28"/>
-      <x:c r="N30" s="37"/>
+      <x:c r="B30" s="28"/>
+      <x:c r="C30" s="28"/>
+      <x:c r="D30" s="8"/>
+      <x:c r="E30" s="12"/>
+      <x:c r="F30" s="8"/>
+      <x:c r="G30" s="12"/>
+      <x:c r="H30" s="12"/>
+      <x:c r="I30" s="8"/>
+      <x:c r="J30" s="8"/>
+      <x:c r="K30" s="24"/>
+      <x:c r="L30" s="25"/>
+      <x:c r="M30" s="26"/>
+      <x:c r="N30" s="35"/>
     </x:row>
     <x:row r="31" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B31" s="30"/>
-      <x:c r="C31" s="30"/>
-      <x:c r="D31" s="10"/>
-      <x:c r="E31" s="14"/>
-      <x:c r="F31" s="10"/>
-      <x:c r="G31" s="14"/>
-      <x:c r="H31" s="14"/>
-      <x:c r="I31" s="10"/>
-      <x:c r="J31" s="10"/>
-      <x:c r="K31" s="26"/>
-      <x:c r="L31" s="27"/>
-      <x:c r="M31" s="28"/>
-      <x:c r="N31" s="37"/>
+      <x:c r="B31" s="28"/>
+      <x:c r="C31" s="28"/>
+      <x:c r="D31" s="8"/>
+      <x:c r="E31" s="12"/>
+      <x:c r="F31" s="8"/>
+      <x:c r="G31" s="12"/>
+      <x:c r="H31" s="12"/>
+      <x:c r="I31" s="8"/>
+      <x:c r="J31" s="8"/>
+      <x:c r="K31" s="24"/>
+      <x:c r="L31" s="25"/>
+      <x:c r="M31" s="26"/>
+      <x:c r="N31" s="35"/>
     </x:row>
     <x:row r="32" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B32" s="30"/>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="10"/>
-      <x:c r="E32" s="14"/>
-      <x:c r="F32" s="10"/>
-      <x:c r="G32" s="14"/>
-      <x:c r="H32" s="14"/>
-      <x:c r="I32" s="10"/>
-      <x:c r="J32" s="10"/>
-      <x:c r="K32" s="26"/>
-      <x:c r="L32" s="36"/>
-      <x:c r="M32" s="28"/>
-      <x:c r="N32" s="37"/>
+      <x:c r="B32" s="28"/>
+      <x:c r="C32" s="28"/>
+      <x:c r="D32" s="8"/>
+      <x:c r="E32" s="12"/>
+      <x:c r="F32" s="8"/>
+      <x:c r="G32" s="12"/>
+      <x:c r="H32" s="12"/>
+      <x:c r="I32" s="8"/>
+      <x:c r="J32" s="8"/>
+      <x:c r="K32" s="24"/>
+      <x:c r="L32" s="34"/>
+      <x:c r="M32" s="26"/>
+      <x:c r="N32" s="35"/>
     </x:row>
     <x:row r="33" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B33" s="38"/>
-      <x:c r="C33" s="38"/>
-      <x:c r="D33" s="10"/>
-      <x:c r="E33" s="14"/>
-      <x:c r="F33" s="10"/>
-      <x:c r="G33" s="14"/>
-      <x:c r="H33" s="14"/>
-      <x:c r="I33" s="10"/>
-      <x:c r="J33" s="10"/>
-      <x:c r="K33" s="26"/>
-      <x:c r="L33" s="36"/>
-      <x:c r="M33" s="28"/>
-      <x:c r="N33" s="37"/>
+      <x:c r="B33" s="36"/>
+      <x:c r="C33" s="36"/>
+      <x:c r="D33" s="8"/>
+      <x:c r="E33" s="12"/>
+      <x:c r="F33" s="8"/>
+      <x:c r="G33" s="12"/>
+      <x:c r="H33" s="12"/>
+      <x:c r="I33" s="8"/>
+      <x:c r="J33" s="8"/>
+      <x:c r="K33" s="24"/>
+      <x:c r="L33" s="34"/>
+      <x:c r="M33" s="26"/>
+      <x:c r="N33" s="35"/>
     </x:row>
     <x:row r="34" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B34" s="30"/>
-      <x:c r="C34" s="30"/>
-      <x:c r="D34" s="10"/>
-      <x:c r="E34" s="14"/>
-      <x:c r="F34" s="10"/>
-      <x:c r="G34" s="14"/>
-      <x:c r="H34" s="14"/>
-      <x:c r="I34" s="10"/>
-      <x:c r="J34" s="10"/>
-      <x:c r="K34" s="26"/>
-      <x:c r="L34" s="36"/>
-      <x:c r="M34" s="28"/>
-      <x:c r="N34" s="37"/>
+      <x:c r="B34" s="28"/>
+      <x:c r="C34" s="28"/>
+      <x:c r="D34" s="8"/>
+      <x:c r="E34" s="12"/>
+      <x:c r="F34" s="8"/>
+      <x:c r="G34" s="12"/>
+      <x:c r="H34" s="12"/>
+      <x:c r="I34" s="8"/>
+      <x:c r="J34" s="8"/>
+      <x:c r="K34" s="24"/>
+      <x:c r="L34" s="34"/>
+      <x:c r="M34" s="26"/>
+      <x:c r="N34" s="35"/>
     </x:row>
     <x:row r="35" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B35" s="38"/>
-      <x:c r="C35" s="38"/>
-      <x:c r="D35" s="10"/>
-      <x:c r="E35" s="10"/>
-      <x:c r="F35" s="10"/>
-      <x:c r="G35" s="14"/>
-      <x:c r="H35" s="14"/>
-      <x:c r="I35" s="10"/>
-      <x:c r="J35" s="10"/>
-      <x:c r="K35" s="26"/>
-      <x:c r="L35" s="36"/>
-      <x:c r="M35" s="28"/>
-      <x:c r="N35" s="37"/>
+      <x:c r="B35" s="36"/>
+      <x:c r="C35" s="36"/>
+      <x:c r="D35" s="8"/>
+      <x:c r="E35" s="8"/>
+      <x:c r="F35" s="8"/>
+      <x:c r="G35" s="12"/>
+      <x:c r="H35" s="12"/>
+      <x:c r="I35" s="8"/>
+      <x:c r="J35" s="8"/>
+      <x:c r="K35" s="24"/>
+      <x:c r="L35" s="34"/>
+      <x:c r="M35" s="26"/>
+      <x:c r="N35" s="35"/>
     </x:row>
     <x:row r="36" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B36" s="30"/>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="10"/>
-      <x:c r="E36" s="14"/>
-      <x:c r="F36" s="10"/>
-      <x:c r="G36" s="14"/>
-      <x:c r="H36" s="14"/>
-      <x:c r="I36" s="10"/>
-      <x:c r="J36" s="10"/>
-      <x:c r="K36" s="26"/>
-      <x:c r="L36" s="36"/>
-      <x:c r="M36" s="28"/>
-      <x:c r="N36" s="37"/>
+      <x:c r="B36" s="28"/>
+      <x:c r="C36" s="28"/>
+      <x:c r="D36" s="8"/>
+      <x:c r="E36" s="12"/>
+      <x:c r="F36" s="8"/>
+      <x:c r="G36" s="12"/>
+      <x:c r="H36" s="12"/>
+      <x:c r="I36" s="8"/>
+      <x:c r="J36" s="8"/>
+      <x:c r="K36" s="24"/>
+      <x:c r="L36" s="34"/>
+      <x:c r="M36" s="26"/>
+      <x:c r="N36" s="35"/>
     </x:row>
     <x:row r="37" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B37" s="30"/>
-      <x:c r="C37" s="30"/>
-      <x:c r="D37" s="30"/>
-      <x:c r="E37" s="38"/>
-      <x:c r="F37" s="30"/>
-      <x:c r="G37" s="38"/>
-      <x:c r="H37" s="38"/>
-      <x:c r="I37" s="30"/>
-      <x:c r="J37" s="30"/>
-      <x:c r="K37" s="42"/>
-      <x:c r="L37" s="43"/>
-      <x:c r="M37" s="44"/>
-      <x:c r="N37" s="45"/>
+      <x:c r="B37" s="28"/>
+      <x:c r="C37" s="28"/>
+      <x:c r="D37" s="28"/>
+      <x:c r="E37" s="36"/>
+      <x:c r="F37" s="28"/>
+      <x:c r="G37" s="36"/>
+      <x:c r="H37" s="36"/>
+      <x:c r="I37" s="28"/>
+      <x:c r="J37" s="28"/>
+      <x:c r="K37" s="40"/>
+      <x:c r="L37" s="41"/>
+      <x:c r="M37" s="42"/>
+      <x:c r="N37" s="43"/>
     </x:row>
     <x:row r="38" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B38" s="30"/>
-      <x:c r="C38" s="30"/>
-      <x:c r="D38" s="30"/>
-      <x:c r="E38" s="30"/>
-      <x:c r="F38" s="30"/>
-      <x:c r="G38" s="38"/>
-      <x:c r="H38" s="38"/>
-      <x:c r="I38" s="30"/>
-      <x:c r="J38" s="30"/>
-      <x:c r="K38" s="42"/>
-      <x:c r="L38" s="43"/>
-      <x:c r="M38" s="44"/>
-      <x:c r="N38" s="45"/>
+      <x:c r="B38" s="28"/>
+      <x:c r="C38" s="28"/>
+      <x:c r="D38" s="28"/>
+      <x:c r="E38" s="28"/>
+      <x:c r="F38" s="28"/>
+      <x:c r="G38" s="36"/>
+      <x:c r="H38" s="36"/>
+      <x:c r="I38" s="28"/>
+      <x:c r="J38" s="28"/>
+      <x:c r="K38" s="40"/>
+      <x:c r="L38" s="41"/>
+      <x:c r="M38" s="42"/>
+      <x:c r="N38" s="43"/>
     </x:row>
     <x:row r="39" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B39" s="30"/>
-      <x:c r="C39" s="30"/>
-      <x:c r="D39" s="30"/>
-      <x:c r="E39" s="30"/>
-      <x:c r="F39" s="30"/>
-      <x:c r="G39" s="38"/>
-      <x:c r="H39" s="38"/>
-      <x:c r="I39" s="30"/>
-      <x:c r="J39" s="30"/>
-      <x:c r="K39" s="42"/>
-      <x:c r="L39" s="43"/>
-      <x:c r="M39" s="44"/>
-      <x:c r="N39" s="46"/>
+      <x:c r="B39" s="28"/>
+      <x:c r="C39" s="28"/>
+      <x:c r="D39" s="28"/>
+      <x:c r="E39" s="28"/>
+      <x:c r="F39" s="28"/>
+      <x:c r="G39" s="36"/>
+      <x:c r="H39" s="36"/>
+      <x:c r="I39" s="28"/>
+      <x:c r="J39" s="28"/>
+      <x:c r="K39" s="40"/>
+      <x:c r="L39" s="41"/>
+      <x:c r="M39" s="42"/>
+      <x:c r="N39" s="44"/>
     </x:row>
     <x:row r="40" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B40" s="30"/>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="38"/>
-      <x:c r="H40" s="38"/>
-      <x:c r="I40" s="30"/>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="42"/>
-      <x:c r="L40" s="43"/>
-      <x:c r="M40" s="42"/>
-      <x:c r="N40" s="47"/>
+      <x:c r="B40" s="28"/>
+      <x:c r="C40" s="28"/>
+      <x:c r="D40" s="28"/>
+      <x:c r="E40" s="28"/>
+      <x:c r="F40" s="28"/>
+      <x:c r="G40" s="36"/>
+      <x:c r="H40" s="36"/>
+      <x:c r="I40" s="28"/>
+      <x:c r="J40" s="28"/>
+      <x:c r="K40" s="40"/>
+      <x:c r="L40" s="41"/>
+      <x:c r="M40" s="40"/>
+      <x:c r="N40" s="45"/>
     </x:row>
     <x:row r="41" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="38"/>
-      <x:c r="H41" s="38"/>
-      <x:c r="I41" s="30"/>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="42"/>
-      <x:c r="L41" s="43"/>
-      <x:c r="M41" s="42"/>
-      <x:c r="N41" s="47"/>
+      <x:c r="B41" s="28"/>
+      <x:c r="C41" s="28"/>
+      <x:c r="D41" s="28"/>
+      <x:c r="E41" s="28"/>
+      <x:c r="F41" s="28"/>
+      <x:c r="G41" s="36"/>
+      <x:c r="H41" s="36"/>
+      <x:c r="I41" s="28"/>
+      <x:c r="J41" s="28"/>
+      <x:c r="K41" s="40"/>
+      <x:c r="L41" s="41"/>
+      <x:c r="M41" s="40"/>
+      <x:c r="N41" s="45"/>
     </x:row>
     <x:row r="42" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B42" s="42"/>
-      <x:c r="C42" s="42"/>
-      <x:c r="D42" s="42"/>
-      <x:c r="E42" s="42"/>
-      <x:c r="F42" s="42"/>
-      <x:c r="G42" s="42"/>
-      <x:c r="H42" s="42"/>
-      <x:c r="I42" s="42"/>
-      <x:c r="J42" s="42"/>
-      <x:c r="K42" s="42"/>
-      <x:c r="L42" s="42"/>
-      <x:c r="M42" s="42"/>
-      <x:c r="N42" s="42"/>
+      <x:c r="B42" s="40"/>
+      <x:c r="C42" s="40"/>
+      <x:c r="D42" s="40"/>
+      <x:c r="E42" s="40"/>
+      <x:c r="F42" s="40"/>
+      <x:c r="G42" s="40"/>
+      <x:c r="H42" s="40"/>
+      <x:c r="I42" s="40"/>
+      <x:c r="J42" s="40"/>
+      <x:c r="K42" s="40"/>
+      <x:c r="L42" s="40"/>
+      <x:c r="M42" s="40"/>
+      <x:c r="N42" s="40"/>
     </x:row>
     <x:row r="43" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B43" s="48"/>
-      <x:c r="C43" s="48"/>
-      <x:c r="D43" s="48"/>
-      <x:c r="E43" s="48"/>
-      <x:c r="F43" s="48"/>
-      <x:c r="G43" s="48"/>
-      <x:c r="H43" s="42"/>
-      <x:c r="I43" s="42"/>
-      <x:c r="J43" s="42"/>
-      <x:c r="K43" s="42"/>
-      <x:c r="L43" s="49"/>
-      <x:c r="M43" s="49"/>
-      <x:c r="N43" s="50"/>
+      <x:c r="B43" s="46"/>
+      <x:c r="C43" s="46"/>
+      <x:c r="D43" s="46"/>
+      <x:c r="E43" s="46"/>
+      <x:c r="F43" s="46"/>
+      <x:c r="G43" s="46"/>
+      <x:c r="H43" s="40"/>
+      <x:c r="I43" s="40"/>
+      <x:c r="J43" s="40"/>
+      <x:c r="K43" s="40"/>
+      <x:c r="L43" s="47"/>
+      <x:c r="M43" s="47"/>
+      <x:c r="N43" s="48"/>
     </x:row>
     <x:row r="44" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B44" s="48"/>
-      <x:c r="C44" s="48"/>
-      <x:c r="D44" s="48"/>
-      <x:c r="E44" s="48"/>
-      <x:c r="F44" s="48"/>
-      <x:c r="G44" s="48"/>
-      <x:c r="H44" s="42"/>
-      <x:c r="K44" s="42"/>
-      <x:c r="L44" s="49"/>
-      <x:c r="M44" s="49"/>
-      <x:c r="N44" s="51"/>
+      <x:c r="B44" s="46"/>
+      <x:c r="C44" s="46"/>
+      <x:c r="D44" s="46"/>
+      <x:c r="E44" s="46"/>
+      <x:c r="F44" s="46"/>
+      <x:c r="G44" s="46"/>
+      <x:c r="H44" s="40"/>
+      <x:c r="K44" s="40"/>
+      <x:c r="L44" s="47"/>
+      <x:c r="M44" s="47"/>
+      <x:c r="N44" s="49"/>
     </x:row>
     <x:row r="45" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B45" s="48"/>
-      <x:c r="C45" s="48"/>
-      <x:c r="D45" s="48"/>
-      <x:c r="E45" s="48"/>
-      <x:c r="F45" s="48"/>
-      <x:c r="G45" s="48"/>
-      <x:c r="H45" s="42"/>
-      <x:c r="I45" s="42"/>
-      <x:c r="J45" s="42"/>
-      <x:c r="K45" s="42"/>
-      <x:c r="L45" s="49"/>
-      <x:c r="M45" s="49"/>
-      <x:c r="N45" s="51"/>
+      <x:c r="B45" s="46"/>
+      <x:c r="C45" s="46"/>
+      <x:c r="D45" s="46"/>
+      <x:c r="E45" s="46"/>
+      <x:c r="F45" s="46"/>
+      <x:c r="G45" s="46"/>
+      <x:c r="H45" s="40"/>
+      <x:c r="I45" s="40"/>
+      <x:c r="J45" s="40"/>
+      <x:c r="K45" s="40"/>
+      <x:c r="L45" s="47"/>
+      <x:c r="M45" s="47"/>
+      <x:c r="N45" s="49"/>
     </x:row>
     <x:row r="46" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B46" s="48"/>
-      <x:c r="C46" s="48"/>
-      <x:c r="D46" s="48"/>
-      <x:c r="E46" s="48"/>
-      <x:c r="F46" s="48"/>
-      <x:c r="G46" s="48"/>
-      <x:c r="H46" s="48"/>
-      <x:c r="I46" s="48"/>
-      <x:c r="J46" s="48"/>
-      <x:c r="K46" s="48"/>
-      <x:c r="L46" s="49"/>
-      <x:c r="M46" s="49"/>
-      <x:c r="N46" s="50"/>
+      <x:c r="B46" s="46"/>
+      <x:c r="C46" s="46"/>
+      <x:c r="D46" s="46"/>
+      <x:c r="E46" s="46"/>
+      <x:c r="F46" s="46"/>
+      <x:c r="G46" s="46"/>
+      <x:c r="H46" s="46"/>
+      <x:c r="I46" s="46"/>
+      <x:c r="J46" s="46"/>
+      <x:c r="K46" s="46"/>
+      <x:c r="L46" s="47"/>
+      <x:c r="M46" s="47"/>
+      <x:c r="N46" s="48"/>
     </x:row>
     <x:row r="47" spans="1:26" ht="112.5" customHeight="1">
-      <x:c r="B47" s="48"/>
-      <x:c r="C47" s="48"/>
-      <x:c r="D47" s="48"/>
-      <x:c r="E47" s="48"/>
-      <x:c r="F47" s="48"/>
-      <x:c r="G47" s="48"/>
-      <x:c r="H47" s="48"/>
-      <x:c r="I47" s="48"/>
-      <x:c r="J47" s="48"/>
-      <x:c r="K47" s="48"/>
-      <x:c r="L47" s="49"/>
-      <x:c r="M47" s="49"/>
-      <x:c r="N47" s="49"/>
+      <x:c r="B47" s="46"/>
+      <x:c r="C47" s="46"/>
+      <x:c r="D47" s="46"/>
+      <x:c r="E47" s="46"/>
+      <x:c r="F47" s="46"/>
+      <x:c r="G47" s="46"/>
+      <x:c r="H47" s="46"/>
+      <x:c r="I47" s="46"/>
+      <x:c r="J47" s="46"/>
+      <x:c r="K47" s="46"/>
+      <x:c r="L47" s="47"/>
+      <x:c r="M47" s="47"/>
+      <x:c r="N47" s="47"/>
     </x:row>
     <x:row r="48" ht="112.5" customHeight="1"/>
     <x:row r="49" ht="112.5" customHeight="1"/>
@@ -3202,7 +3374,7 @@
     <x:row r="999" ht="12.75" customHeight="1"/>
     <x:row r="1000" ht="12.75" customHeight="1"/>
   </x:sheetData>
-  <x:mergeCells count="32">
+  <x:mergeCells count="37">
     <x:mergeCell ref="B8:G8"/>
     <x:mergeCell ref="J8:N8"/>
     <x:mergeCell ref="B9:H9"/>
@@ -3226,6 +3398,11 @@
     <x:mergeCell ref="G15:I15"/>
     <x:mergeCell ref="J15:N15"/>
     <x:mergeCell ref="B16:N16"/>
+    <x:mergeCell ref="B20:G20"/>
+    <x:mergeCell ref="H20:J20"/>
+    <x:mergeCell ref="K20:L20"/>
+    <x:mergeCell ref="K21:L21"/>
+    <x:mergeCell ref="K22:L22"/>
     <x:mergeCell ref="D28:D29"/>
     <x:mergeCell ref="E28:E29"/>
     <x:mergeCell ref="F28:F29"/>
@@ -3237,10 +3414,10 @@
     <x:mergeCell ref="N28:N29"/>
   </x:mergeCells>
   <x:printOptions horizontalCentered="1" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <x:pageSetup paperSize="9" pageOrder="downThenOver" orientation="landscape" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:pageMargins left="0.3937007874015748" right="0.3937007874015748" top="0.3937007874015748" bottom="0.3937007874015748" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <x:pageSetup paperSize="9" pageOrder="downThenOver" orientation="landscape" blackAndWhite="0" draft="0" cellComments="none" errors="displayed" r:id="rId1"/>
   <x:headerFooter/>
-  <x:drawing r:id="rId1"/>
+  <x:drawing r:id="rId2"/>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
@@ -3265,90 +3442,90 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:26" ht="15" customHeight="1">
-      <x:c r="B1" s="112" t="s">
+      <x:c r="B1" s="125" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C1" s="126" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D1" s="126" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C1" s="113" t="s">
+      <x:c r="E1" s="126" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D1" s="113" t="s">
+      <x:c r="F1" s="125" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G1" s="125" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E1" s="113" t="s">
+      <x:c r="H1" s="125" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F1" s="112" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G1" s="112" t="s">
+      <x:c r="I1" s="126" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="H1" s="112" t="s">
+      <x:c r="J1" s="50" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="I1" s="113" t="s">
+      <x:c r="K1" s="50" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="J1" s="52" t="s">
+      <x:c r="L1" s="50" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="K1" s="52" t="s">
+    </x:row>
+    <x:row r="2" spans="1:26" ht="15" customHeight="1">
+      <x:c r="B2" s="50" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C2" s="50" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="L1" s="52" t="s">
+      <x:c r="D2" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E2" s="53" t="s">
         <x:v>34</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:26" ht="15" customHeight="1">
-      <x:c r="B2" s="52" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C2" s="52" t="s">
+      <x:c r="F2" s="50" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="G2" s="50" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="H2" s="50" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="D2" s="52" t="s">
+      <x:c r="I2" s="50" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="J2" s="50" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="E2" s="55" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F2" s="52" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G2" s="52" t="s">
+      <x:c r="K2" s="50" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="L2" s="50" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="H2" s="52" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="I2" s="52" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J2" s="52" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="K2" s="52" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="L2" s="52" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="M2" s="52" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="N2" s="52" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="O2" s="52" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="P2" s="52" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="Q2" s="52"/>
-      <x:c r="R2" s="52"/>
-      <x:c r="S2" s="52"/>
-      <x:c r="Z2" s="52"/>
+      <x:c r="M2" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="N2" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="O2" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="P2" s="50" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="Q2" s="50"/>
+      <x:c r="R2" s="50"/>
+      <x:c r="S2" s="50"/>
+      <x:c r="Z2" s="50"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>